<commit_message>
Aylık OFÖ verileri güncellendi: 2026-08-18
</commit_message>
<xml_diff>
--- a/OFO_Faiz_Oranlari.xlsx
+++ b/OFO_Faiz_Oranlari.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -509,6 +509,276 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Akbank (Axess)</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Sayfada faiz verisi var (Detay için linke bakınız)</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Sayfada ücret/masraf verisi var (Detay için linke bakınız)</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Garanti BBVA</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Sayfada faiz verisi var (Detay için linke bakınız)</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Sayfada ücret/masraf verisi var (Detay için linke bakınız)</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Yapı Kredi</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Sayfada faiz verisi var (Detay için linke bakınız)</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Sayfada ücret/masraf verisi var (Detay için linke bakınız)</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>İş Bankası</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Sayfada faiz verisi var (Detay için linke bakınız)</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Sayfada ücret/masraf verisi var (Detay için linke bakınız)</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>DenizBank</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Sayfada faiz verisi var (Detay için linke bakınız)</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Sayfada ücret/masraf verisi var (Detay için linke bakınız)</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>QNB</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Faiz verisi tespit edilemedi</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Ücret verisi tespit edilemedi</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>TEB</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Sayfada faiz verisi var (Detay için linke bakınız)</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Sayfada ücret/masraf verisi var (Detay için linke bakınız)</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Halkbank</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Sayfada faiz verisi var (Detay için linke bakınız)</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Sayfada ücret/masraf verisi var (Detay için linke bakınız)</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>VakıfBank</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Sayfada faiz verisi var (Detay için linke bakınız)</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Sayfada ücret/masraf verisi var (Detay için linke bakınız)</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Ziraat Bankası</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Faiz verisi tespit edilemedi</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Ücret verisi tespit edilemedi</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>